<commit_message>
docs(order-history): resolve 13.2 order-listing open questions + add implementation plan
- Resolve order-scope open question: GET /orders spans all three order types
  (product, subscription, ppl_addon) from the single orders table; shows[] empty
  (not null) for non-product orders
- Add pending-orders open question (direction: include) for team discussion
- Add invoice-semantics open question (A: per-order PDF vs B: persisted rows);
  defer the invoice endpoint (13.2-g) until the team confirms
- Add Deferred Work section to the feasibility doc
- Sync the same resolutions into the .xlsx Open Questions sheet (new Status +
  Resolution columns)
- Add the 13.2 implementation plan (GET /orders listing) alongside the
  feasibility docs
</commit_message>
<xml_diff>
--- a/order_history/13.2-order-listing-table/13.2 - Order Listing Table.xlsx
+++ b/order_history/13.2-order-listing-table/13.2 - Order Listing Table.xlsx
@@ -1623,11 +1623,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="120" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="120" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1641,6 +1643,16 @@
           <t>Open Question</t>
         </is>
       </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>Resolution / Decision</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -1648,7 +1660,57 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Does 'all the Exhibitor's orders' include PPL subscription/ppl_addon orders (which have no showProduct and would render an empty 'Associated Shows' column), or is the listing limited to product/booth (show) orders? Today these are listed by two different, non-overlapping paths — ppl.service.listOrderHistory filters to subscription/ppl_addon only and explicitly EXCLUDES product orders, while purchased-booths filters to product/show orders only — so the unified scope of this new listing is a genuine product decision.</t>
+          <t>[RESOLVED 2026-06-30] Does 'all the Exhibitor's orders' include PPL subscription/ppl_addon orders (which have no showProduct and would render an empty 'Associated Shows' column), or is the listing limited to product/booth (show) orders? Today these are listed by two different, non-overlapping paths — ppl.service.listOrderHistory filters to subscription/ppl_addon only and explicitly EXCLUDES product orders, while purchased-booths filters to product/show orders only — so the unified scope of this new listing is a genuine product decision.</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Resolved (2026-06-30)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Decision: GET /orders spans ALL THREE order types (product, subscription, ppl_addon) from the single orders table — no order_type narrowing. All orders live in one Order model (admin-backend-api/prisma/schema.prisma:1540; order_type enum at :1545); the existing PPL and purchased-booths pages differ only by their order_type filter, so the unified listing relaxes that predicate. Consequence: Associated Shows renders only for product orders (orderItems -&gt; showProduct -&gt; show) and is an empty array for subscription/ppl_addon orders, which the row DTO returns as shows: [] (not null).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Should abandoned pending orders appear in the listing? A pending Order row is written at place-order time (before the Stripe redirect); if the exhibitor backs out it stays pending forever. The existing PPL history deliberately excludes pending and shows only terminal/active states.</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Open — for team discussion</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Current direction (2026-06-30): INCLUDE pending rows in GET /orders so in-flight/current orders surface (consistent with 13.1 past-AND-current mandate and the Pay action on payable orders). Flagged for TEAM DISCUSSION because this also surfaces never-paid abandoned-checkout rows, which may add noise; team to decide whether to keep, filter by an age cutoff, or exclude pure abandoned-checkout pending orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>What does the Invoice action mean for the listing — a formal tax invoice/receipt for money actually paid, or an order document/summary downloadable regardless of payment state? Current invoice generation is PPL/subscription-only: the Stripe webhook persists Invoice+InvoiceLineItem rows ONLY on successful payment (unpaid order -&gt; 0 invoices; split order -&gt; N invoices), and the single PDF renderer (ppl.service.ts:985 renderInvoicePdf, pdfkit, GET /ppl/invoices/:id/download) is hardcoded subscription-shaped and cannot render product/booth orders as-is. No product-order invoice renderer exists.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Open — team confirmation · work DEFERRED</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Decision (2026-06-30): DEFER the Invoice endpoint work (13.2-g, GET /orders/:orderId/invoice) until the team confirms invoice semantics. Option A: generate an order-level invoice/summary PDF from Order+OrderItems (works for every order &amp; payment state). Option B: serve only persisted Invoice rows (unpaid -&gt; 404, split -&gt; latest-vs-all ambiguity, still needs a product-shaped renderer). The listing endpoint and all other rows/actions proceed now; the invoice PDF endpoint and Invoice action-availability flag are HELD pending this answer.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(order-history): record 13.2 implementation status
Add implementation status to the 13.2 story feasibility docs (.md + .xlsx):
12 of 13 in-scope requirements shipped in SBE-1146 (GET /orders listing),
with 13.2-g (Invoice action/endpoint) remaining — deferred pending the
team's invoice-semantics decision. Notes the open pending-orders decision
and the 13.3 / 13.2-h2 dependencies owned by other stories.
</commit_message>
<xml_diff>
--- a/order_history/13.2-order-listing-table/13.2 - Order Listing Table.xlsx
+++ b/order_history/13.2-order-listing-table/13.2 - Order Listing Table.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Endpoints" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Open Questions" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Cross-Epic Dependencies" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Implementation Status" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Requirements'!$A$1:$K$15</definedName>
@@ -112,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -148,6 +149,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -515,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -654,6 +661,54 @@
       </c>
       <c r="B13" s="8" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Implementation</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>12 of 13 in-scope reqs shipped in SBE-1146; 13.2-g Invoice DEFERRED (team decision)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Impl Branch</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>feature/SBE-1146-order-listing-table (exhibitor-backend-api)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Impl Commits</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>09bce5f (feat), fc429bd (SonarQube fix)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Bitbucket #272 → dev</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -667,7 +722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -681,6 +736,7 @@
     <col width="48" customWidth="1" min="9" max="9"/>
     <col width="62" customWidth="1" min="10" max="10"/>
     <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="46" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -739,6 +795,11 @@
           <t>Confluence</t>
         </is>
       </c>
+      <c r="L1" s="9" t="inlineStr">
+        <is>
+          <t>Impl Status (2026-07-01)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -790,6 +851,11 @@
       <c r="K2" s="10" t="inlineStr">
         <is>
           <t>Open §Order History → Story 13.2</t>
+        </is>
+      </c>
+      <c r="L2" s="13" t="inlineStr">
+        <is>
+          <t>✅ Done (SBE-1146)</t>
         </is>
       </c>
     </row>
@@ -841,6 +907,11 @@
           <t>Open §Order History → Story 13.2</t>
         </is>
       </c>
+      <c r="L3" s="13" t="inlineStr">
+        <is>
+          <t>✅ Done (SBE-1146)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -892,6 +963,11 @@
       <c r="K4" s="10" t="inlineStr">
         <is>
           <t>Open §Order History → Story 13.2</t>
+        </is>
+      </c>
+      <c r="L4" s="13" t="inlineStr">
+        <is>
+          <t>✅ Done (SBE-1146)</t>
         </is>
       </c>
     </row>
@@ -943,6 +1019,11 @@
           <t>Open §Order History → Story 13.2</t>
         </is>
       </c>
+      <c r="L5" s="13" t="inlineStr">
+        <is>
+          <t>✅ Done (SBE-1146) — order-level is_overdue rollup; per-installment breakdown = 13.3</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -996,6 +1077,11 @@
           <t>Open §Order History → Story 13.2</t>
         </is>
       </c>
+      <c r="L6" s="13" t="inlineStr">
+        <is>
+          <t>✅ Done (SBE-1146)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1053,6 +1139,11 @@
           <t>Open §Order History → Story 13.2</t>
         </is>
       </c>
+      <c r="L7" s="13" t="inlineStr">
+        <is>
+          <t>✅ Done (SBE-1146) — row id returned; details endpoint owned by 13.3</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1104,6 +1195,11 @@
       <c r="K8" s="10" t="inlineStr">
         <is>
           <t>Open §Order History → Story 13.2</t>
+        </is>
+      </c>
+      <c r="L8" s="13" t="inlineStr">
+        <is>
+          <t>⛔ DEFERRED — Invoice endpoint + action flag; blocked on team invoice-semantics decision (A vs B)</t>
         </is>
       </c>
     </row>
@@ -1155,6 +1251,11 @@
           <t>Open §Order History → Story 13.2</t>
         </is>
       </c>
+      <c r="L9" s="13" t="inlineStr">
+        <is>
+          <t>⚠️ Partial (SBE-1146) — Pay flag + View shipped; Invoice action flag deferred with 13.2-g</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1206,6 +1307,11 @@
       <c r="K10" s="10" t="inlineStr">
         <is>
           <t>Open §Order History → Story 13.2</t>
+        </is>
+      </c>
+      <c r="L10" s="13" t="inlineStr">
+        <is>
+          <t>Out of Scope — Credit Card Payment Workflow / Payment Schedule Visibility stories</t>
         </is>
       </c>
     </row>
@@ -1257,6 +1363,11 @@
           <t>Open §Order History → Story 13.2</t>
         </is>
       </c>
+      <c r="L11" s="13" t="inlineStr">
+        <is>
+          <t>✅ Done (SBE-1146)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1310,6 +1421,11 @@
           <t>Open §Order History → Story 13.2</t>
         </is>
       </c>
+      <c r="L12" s="13" t="inlineStr">
+        <is>
+          <t>✅ Done (SBE-1146)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1361,6 +1477,11 @@
       <c r="K13" s="10" t="inlineStr">
         <is>
           <t>Open §Order History → Story 13.2</t>
+        </is>
+      </c>
+      <c r="L13" s="13" t="inlineStr">
+        <is>
+          <t>✅ Done (SBE-1146)</t>
         </is>
       </c>
     </row>
@@ -1412,6 +1533,11 @@
           <t>Open §Order History → Story 13.2</t>
         </is>
       </c>
+      <c r="L14" s="13" t="inlineStr">
+        <is>
+          <t>✅ Done (SBE-1146)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1463,6 +1589,11 @@
       <c r="K15" s="10" t="inlineStr">
         <is>
           <t>Open §Order History → Story 13.2</t>
+        </is>
+      </c>
+      <c r="L15" s="13" t="inlineStr">
+        <is>
+          <t>✅ Done (SBE-1146)</t>
         </is>
       </c>
     </row>
@@ -1787,4 +1918,118 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="B1" s="14" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>Shipped (SBE-1146)</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>GET /orders listing endpoint (src/orders/) — satisfies 12 of 13 in-scope reqs: 13.2-a,b,c,d,e,f,h(Pay+View),i,j,k,l,m. Exposed in Swagger under the Orders tag. Live-smoke-tested, code-reviewed, pre-push gate green.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>Remaining — 13.2-g</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Invoice action + endpoint GET /orders/:orderId/invoice AND the Invoice action-availability flag (Invoice half of 13.2-h). DEFERRED — blocked on team invoice-semantics decision: Option A (order-level PDF from Order+OrderItems, works for every order/state) vs Option B (serve persisted Invoice rows). Only piece of 13.2 own backend not yet built.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Open decision — invoice semantics</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>A vs B — gates 13.2-g. No code until answered.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Open decision — pending orders</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Currently SHIPPED as included; team to confirm keep / age-filter / exclude abandoned-checkout pending (single where predicate if changed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Dependency — 13.3</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>GET /orders/:orderId order-details aggregate owned by story 13.3 (View navigation target; 13.2 only owes the row id, which is shipped).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>Dependency — 13.2-h2</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Pay-flow execution (Out of Scope) — Credit Card Payment Workflow / Payment Schedule Visibility stories.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Out of API scope</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Front-end row-to-detail / action wiring.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>